<commit_message>
DSA: Update strip_meta() and include inside rename_trollcols() wrapper
</commit_message>
<xml_diff>
--- a/inst/Functions_list.xlsx
+++ b/inst/Functions_list.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>Function Name</t>
   </si>
@@ -37,6 +37,18 @@
   </si>
   <si>
     <t>depth_rounder()</t>
+  </si>
+  <si>
+    <t>troll_run_stats()</t>
+  </si>
+  <si>
+    <t>is_stationary()</t>
+  </si>
+  <si>
+    <t>remove_jiggle()</t>
+  </si>
+  <si>
+    <t>troll_rollRange()</t>
   </si>
 </sst>
 </file>
@@ -386,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -422,6 +434,29 @@
         <v>6</v>
       </c>
     </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>